<commit_message>
Phase 3 통합시험: 강제해제(P2) > 접근위험(P3) > ISOFIX(P4) > ignition-off(P5) 우선순위 검증
함수커버리지 100%, 콜커버리지 100%.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02_Tier/02_WorkProduct/doc/engineering/SoftwareComponentVerificationAndIntegrationVerification/ENG-SWE5-002_SW 통합시험 케이스.xlsx
+++ b/02_Tier/02_WorkProduct/doc/engineering/SoftwareComponentVerificationAndIntegrationVerification/ENG-SWE5-002_SW 통합시험 케이스.xlsx
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1085,6 +1085,228 @@
         </is>
       </c>
       <c r="G18" t="inlineStr">
+        <is>
+          <t>자동(unittest)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>IT-P3-01</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>SWR-017</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>ForcedReleasePolicy+InputGateway</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>fire_detected=True</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>RELEASE</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>요구사항기반시험</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>자동(unittest)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>IT-P3-02</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>SWR-017, SWR-005</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>ForcedReleasePolicy+ApproachRiskPolicy</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>화재=True, 접근위험=True 동시</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>RELEASE (P2&gt;P3)</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>의사결정표기반</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>자동(unittest)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>IT-P3-03</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>SWR-018, SWR-020</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>IsofixLockPolicy+IgnitionOffPolicy</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>isofix_left=True, ignition_on=False 동시</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LOCK (P4&gt;P5)</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>의사결정표기반</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>자동(unittest)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>IT-P3-04</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>SWR-007, SWR-017</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>CrashReleasePolicy+ForcedReleasePolicy</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>crash_status=CONFIRMED, fire_detected=True 동시</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>RELEASE (동일결과 일관성)</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>요구사항기반시험</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>자동(unittest)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>IT-P3-05</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>SWR-021, SWR-017, SWR-018</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>SensorFaultGate+ForcedReleasePolicy+IsofixLockPolicy</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>sensor_fault=True, fire_detected=True, isofix_left=True</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>HOLD_LAST_OUTPUT (P0 최우선)</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>결함주입시험</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>자동(unittest)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>IT-P3-06</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>전체</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Phase1~3 전체 정책</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>모든 트리거 False</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>vote 없음</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>요구사항기반시험</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
         <is>
           <t>자동(unittest)</t>
         </is>

</xml_diff>

<commit_message>
Phase 3 통합시험: 우선순위 P2>P3>P4>P5 검증 (#15)
함수커버리지 100%, 콜커버리지 100%.

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02_Tier/02_WorkProduct/doc/engineering/SoftwareComponentVerificationAndIntegrationVerification/ENG-SWE5-002_SW 통합시험 케이스.xlsx
+++ b/02_Tier/02_WorkProduct/doc/engineering/SoftwareComponentVerificationAndIntegrationVerification/ENG-SWE5-002_SW 통합시험 케이스.xlsx
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1085,6 +1085,228 @@
         </is>
       </c>
       <c r="G18" t="inlineStr">
+        <is>
+          <t>자동(unittest)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>IT-P3-01</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>SWR-017</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>ForcedReleasePolicy+InputGateway</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>fire_detected=True</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>RELEASE</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>요구사항기반시험</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>자동(unittest)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>IT-P3-02</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>SWR-017, SWR-005</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>ForcedReleasePolicy+ApproachRiskPolicy</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>화재=True, 접근위험=True 동시</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>RELEASE (P2&gt;P3)</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>의사결정표기반</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>자동(unittest)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>IT-P3-03</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>SWR-018, SWR-020</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>IsofixLockPolicy+IgnitionOffPolicy</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>isofix_left=True, ignition_on=False 동시</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LOCK (P4&gt;P5)</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>의사결정표기반</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>자동(unittest)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>IT-P3-04</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>SWR-007, SWR-017</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>CrashReleasePolicy+ForcedReleasePolicy</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>crash_status=CONFIRMED, fire_detected=True 동시</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>RELEASE (동일결과 일관성)</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>요구사항기반시험</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>자동(unittest)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>IT-P3-05</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>SWR-021, SWR-017, SWR-018</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>SensorFaultGate+ForcedReleasePolicy+IsofixLockPolicy</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>sensor_fault=True, fire_detected=True, isofix_left=True</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>HOLD_LAST_OUTPUT (P0 최우선)</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>결함주입시험</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>자동(unittest)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>IT-P3-06</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>전체</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Phase1~3 전체 정책</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>모든 트리거 False</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>vote 없음</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>요구사항기반시험</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
         <is>
           <t>자동(unittest)</t>
         </is>

</xml_diff>